<commit_message>
Refine visual design based on feedback
</commit_message>
<xml_diff>
--- a/docs/prototype_evaluation_test_cases.xlsx
+++ b/docs/prototype_evaluation_test_cases.xlsx
@@ -4,11 +4,12 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="24030" windowHeight="10080"/>
+    <workbookView windowWidth="20690" windowHeight="9470"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
     <sheet name="Requirement Checklist" sheetId="2" r:id="rId2"/>
+    <sheet name="Boundary Tests" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="270">
   <si>
     <t>Test ID</t>
   </si>
@@ -735,17 +736,212 @@
   <si>
     <t>Future integration with DLC backend/CMS</t>
   </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>Expected Behavior</t>
+  </si>
+  <si>
+    <t>Observed Behavior</t>
+  </si>
+  <si>
+    <t>Limitation / Future Handling</t>
+  </si>
+  <si>
+    <t>TC16</t>
+  </si>
+  <si>
+    <t>Test layout behavior with a very short title.</t>
+  </si>
+  <si>
+    <t>KI Basics</t>
+  </si>
+  <si>
+    <t>10:00–12:00</t>
+  </si>
+  <si>
+    <t>https://dlc.sh/</t>
+  </si>
+  <si>
+    <t>A short introductory learning offer about
+ artificial intelligence and its practical use in everyday work.</t>
+  </si>
+  <si>
+    <t>The assets are generated successfully. 
+The short title remains readable and the layout still looks balanced.</t>
+  </si>
+  <si>
+    <t>Generated successfully; layout has more empty space but remains readable.</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Very short titles may leave unused space. 
+Future templates could adjust title positioning dynamically.</t>
+  </si>
+  <si>
+    <t>TC17</t>
+  </si>
+  <si>
+    <t>Test layout behavior with a very long learning-offer title.</t>
+  </si>
+  <si>
+    <t>Digitale Kompetenzen für nachhaltige 
+Projektarbeit in Bildung, Verwaltung und gemeinnützigen Organisationen</t>
+  </si>
+  <si>
+    <t>14:00–17:00</t>
+  </si>
+  <si>
+    <t>Mittelstufe</t>
+  </si>
+  <si>
+    <t>This learning offer introduces practical 
+digital tools and methods for planning, communication, collaboration, and documentation in project-based work.</t>
+  </si>
+  <si>
+    <t>The title is wrapped or shortened 
+without breaking the overall layout. The QR code and metadata remain visible.</t>
+  </si>
+  <si>
+    <t>Generation successful; 
+the title spans multiple lines, but only three lines of content are displayed.</t>
+  </si>
+  <si>
+    <t>Very long titles may require a smaller 
+font size, stricter character limits, or alternative title layouts.</t>
+  </si>
+  <si>
+    <t>TC18</t>
+  </si>
+  <si>
+    <t>Test layout behavior with an extremely long single word in
+ the title.</t>
+  </si>
+  <si>
+    <t>Digitalisierungskompetenzentwicklungsworkshop</t>
+  </si>
+  <si>
+    <t>09:30–11:30</t>
+  </si>
+  <si>
+    <t>A workshop about developing digital skills 
+through practical exercises, examples, and guided reflection.</t>
+  </si>
+  <si>
+    <t>The output is generated without 
+crashing.The long word should remain visible, although it may not wrap ideally.</t>
+  </si>
+  <si>
+    <t>Generated successfully;
+long word does not wrap optimally and may require manual layout adjustment.</t>
+  </si>
+  <si>
+    <t>Long compound words may require hyphenation, 
+automatic font scaling, or forced line breaking.</t>
+  </si>
+  <si>
+    <t>TC19</t>
+  </si>
+  <si>
+    <t>Test handling of a very long description.</t>
+  </si>
+  <si>
+    <t>Digitale Werkzeuge im Arbeitsalltag</t>
+  </si>
+  <si>
+    <t>13:00–16:00</t>
+  </si>
+  <si>
+    <t>In diesem Lernangebot erhalten Teilnehmende
+ einen praxisnahen Überblick über digitale Werkzeuge für Kommunikation, Zusammenarbeit, Aufgabenmanagement und Dokumentation. Anhand konkreter Beispiele wird gezeigt, wie digitale Anwendungen sinnvoll in den Arbeitsalltag integriert werden können. Der Kurs richtet sich an Personen, die ihre digitalen Kompetenzen erweitern möchten und nach einfachen, verständlichen und direkt anwendbaren Methoden suchen. Zusätzlich werden typische Herausforderungen wie Datenschutz, Informationsflut und die Auswahl geeigneter Tools diskutiert.</t>
+  </si>
+  <si>
+    <t>The full description is saved in 
+metadata and press text, while image-based assets use a shortened version without layout overflow.</t>
+  </si>
+  <si>
+    <t>Generated successfully;
+social media post and flyer show shortened description; press text keeps full description.</t>
+  </si>
+  <si>
+    <t>Long official descriptions are not ideal for 
+visual assets. DLC could provide additional teaser_text or promotional_description metadata.</t>
+  </si>
+  <si>
+    <t>TC20</t>
+  </si>
+  <si>
+    <t>Test German umlauts, punctuation, and special characters.</t>
+  </si>
+  <si>
+    <t>Einführung in KI: Chancen, Risiken &amp;
+ praktische Übungen</t>
+  </si>
+  <si>
+    <t>15:00–18:00</t>
+  </si>
+  <si>
+    <t>Wie verändert Künstliche Intelligenz unseren
+Alltag?🎧In diesem Angebot geht es um Möglichkeiten, Grenzen, Datenschutz-Fragen und praktische Beispiele für Schule, Beruf und Ehrenamt. Teilnehmende können Fragen stellen und erste Tools ausprobieren.</t>
+  </si>
+  <si>
+    <t>German umlauts and punctuation are 
+rendered correctly. Unsupported symbols should not crash the image generation.</t>
+  </si>
+  <si>
+    <t>Generation successful; 
+German characters display correctly. Emojis are automatically removed from posts and flyers.</t>
+  </si>
+  <si>
+    <t>Additional multilingual testing is required 
+for non-Latin scripts or mixed-language typesetting. Additionally, emojis need to be included in the post.</t>
+  </si>
+  <si>
+    <t>TVC21</t>
+  </si>
+  <si>
+    <t>Test behavior with missing optional metadata fields.</t>
+  </si>
+  <si>
+    <t>Offene Beratung zu digitalen Kompetenzen</t>
+  </si>
+  <si>
+    <t>An open consultation format for learners 
+who want to ask questions about digital tools, online services, and everyday digital challenges.</t>
+  </si>
+  <si>
+    <t>The prototype still generates assets 
+because title and URL are present. Empty date and time fields may appear blank in the output.</t>
+  </si>
+  <si>
+    <t>Generated successfully; 
+date/time area is empty, which reduces clarity.</t>
+  </si>
+  <si>
+    <t>Missing metadata should be handled with 
+placeholders such as “Date to be announced” or validation warnings.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="d\ mmm\ yyyy"/>
+    <numFmt numFmtId="176" formatCode="d\ mmmm\ yyyy"/>
+    <numFmt numFmtId="177" formatCode="d\ mmm\ yyyy"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -758,7 +954,7 @@
     <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF0000FF"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -766,7 +962,7 @@
     <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF800080"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1220,10 +1416,10 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
@@ -1354,20 +1550,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1909,7 +2105,7 @@
     <col min="1" max="1" width="11.5454545454545" customWidth="1"/>
     <col min="2" max="2" width="56.6363636363636" customWidth="1"/>
     <col min="3" max="3" width="39.7272727272727" customWidth="1"/>
-    <col min="4" max="4" width="18.6363636363636" style="2" customWidth="1"/>
+    <col min="4" max="4" width="18.6363636363636" style="5" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="17.5454545454545" customWidth="1"/>
     <col min="7" max="7" width="15.9090909090909" customWidth="1"/>
@@ -1932,7 +2128,7 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
@@ -1976,10 +2172,10 @@
       <c r="B2" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="5">
         <v>46155</v>
       </c>
       <c r="E2" t="s">
@@ -1994,7 +2190,7 @@
       <c r="H2" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="3" t="s">
         <v>22</v>
       </c>
       <c r="J2" t="s">
@@ -2009,10 +2205,10 @@
       <c r="M2" t="s">
         <v>26</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="3" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2023,10 +2219,10 @@
       <c r="B3" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="5">
         <v>46156</v>
       </c>
       <c r="E3" t="s">
@@ -2041,7 +2237,7 @@
       <c r="H3" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="3" t="s">
         <v>34</v>
       </c>
       <c r="J3" t="s">
@@ -2053,13 +2249,13 @@
       <c r="L3" t="s">
         <v>37</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="N3" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="O3" s="3" t="s">
         <v>40</v>
       </c>
     </row>
@@ -2070,10 +2266,10 @@
       <c r="B4" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="5">
         <v>46157</v>
       </c>
       <c r="E4" t="s">
@@ -2100,13 +2296,13 @@
       <c r="L4" t="s">
         <v>48</v>
       </c>
-      <c r="M4" s="4" t="s">
+      <c r="M4" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="N4" s="4" t="s">
+      <c r="N4" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="O4" s="4" t="s">
+      <c r="O4" s="3" t="s">
         <v>50</v>
       </c>
     </row>
@@ -2117,13 +2313,13 @@
       <c r="B5" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="5">
         <v>46159</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>54</v>
       </c>
       <c r="F5" t="s">
@@ -2135,7 +2331,7 @@
       <c r="H5" t="s">
         <v>21</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="3" t="s">
         <v>56</v>
       </c>
       <c r="J5" t="s">
@@ -2150,10 +2346,10 @@
       <c r="M5" t="s">
         <v>26</v>
       </c>
-      <c r="N5" s="4" t="s">
+      <c r="N5" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="O5" s="4" t="s">
+      <c r="O5" s="3" t="s">
         <v>59</v>
       </c>
     </row>
@@ -2161,28 +2357,28 @@
       <c r="A6" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C6" t="s">
         <v>62</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="5">
         <v>46160</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="3" t="s">
         <v>63</v>
       </c>
       <c r="F6" t="s">
         <v>64</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="3" t="s">
         <v>20</v>
       </c>
       <c r="H6" t="s">
         <v>21</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="3" t="s">
         <v>65</v>
       </c>
       <c r="J6" t="s">
@@ -2197,10 +2393,10 @@
       <c r="M6" t="s">
         <v>26</v>
       </c>
-      <c r="N6" s="4" t="s">
+      <c r="N6" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="O6" s="4" t="s">
+      <c r="O6" s="3" t="s">
         <v>68</v>
       </c>
     </row>
@@ -2211,10 +2407,10 @@
       <c r="B7" t="s">
         <v>70</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="5">
         <v>46161</v>
       </c>
       <c r="E7" t="s">
@@ -2223,13 +2419,13 @@
       <c r="F7" t="s">
         <v>19</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="3" t="s">
         <v>20</v>
       </c>
       <c r="H7" t="s">
         <v>21</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="3" t="s">
         <v>73</v>
       </c>
       <c r="J7" t="s">
@@ -2247,7 +2443,7 @@
       <c r="N7" t="s">
         <v>76</v>
       </c>
-      <c r="O7" s="4" t="s">
+      <c r="O7" s="3" t="s">
         <v>77</v>
       </c>
     </row>
@@ -2261,7 +2457,7 @@
       <c r="C8" t="s">
         <v>80</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="5" t="s">
         <v>81</v>
       </c>
       <c r="E8" t="s">
@@ -2276,7 +2472,7 @@
       <c r="H8" t="s">
         <v>21</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="3" t="s">
         <v>83</v>
       </c>
       <c r="J8" t="s">
@@ -2294,7 +2490,7 @@
       <c r="N8" t="s">
         <v>76</v>
       </c>
-      <c r="O8" s="4" t="s">
+      <c r="O8" s="3" t="s">
         <v>84</v>
       </c>
     </row>
@@ -2308,7 +2504,7 @@
       <c r="C9" t="s">
         <v>87</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="5">
         <v>46160</v>
       </c>
       <c r="E9" t="s">
@@ -2323,7 +2519,7 @@
       <c r="H9" t="s">
         <v>21</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="3" t="s">
         <v>89</v>
       </c>
       <c r="J9" t="s">
@@ -2338,10 +2534,10 @@
       <c r="M9" t="s">
         <v>26</v>
       </c>
-      <c r="N9" s="4" t="s">
+      <c r="N9" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="O9" s="4" t="s">
+      <c r="O9" s="3" t="s">
         <v>92</v>
       </c>
     </row>
@@ -2352,10 +2548,10 @@
       <c r="B10" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="5" t="s">
         <v>81</v>
       </c>
       <c r="E10" t="s">
@@ -2370,7 +2566,7 @@
       <c r="H10" t="s">
         <v>21</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="3" t="s">
         <v>97</v>
       </c>
       <c r="J10" t="s">
@@ -2388,7 +2584,7 @@
       <c r="N10" t="s">
         <v>76</v>
       </c>
-      <c r="O10" s="4" t="s">
+      <c r="O10" s="3" t="s">
         <v>99</v>
       </c>
     </row>
@@ -2399,10 +2595,10 @@
       <c r="B11" t="s">
         <v>101</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="5">
         <v>46160</v>
       </c>
       <c r="E11" t="s">
@@ -2417,7 +2613,7 @@
       <c r="H11" t="s">
         <v>21</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="I11" s="3" t="s">
         <v>104</v>
       </c>
       <c r="J11" t="s">
@@ -2432,7 +2628,7 @@
       <c r="M11" t="s">
         <v>26</v>
       </c>
-      <c r="N11" s="4" t="s">
+      <c r="N11" s="3" t="s">
         <v>108</v>
       </c>
       <c r="O11" t="s">
@@ -2446,10 +2642,10 @@
       <c r="B12" t="s">
         <v>111</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="5">
         <v>46161</v>
       </c>
       <c r="E12" t="s">
@@ -2464,7 +2660,7 @@
       <c r="H12" t="s">
         <v>21</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="3" t="s">
         <v>114</v>
       </c>
       <c r="J12" t="s">
@@ -2487,13 +2683,13 @@
       <c r="A13" t="s">
         <v>116</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="5">
         <v>46162</v>
       </c>
       <c r="E13" t="s">
@@ -2508,7 +2704,7 @@
       <c r="H13" t="s">
         <v>21</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="I13" s="3" t="s">
         <v>120</v>
       </c>
       <c r="J13" t="s">
@@ -2534,10 +2730,10 @@
       <c r="B14" t="s">
         <v>124</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="5">
         <v>46162</v>
       </c>
       <c r="E14" t="s">
@@ -2552,7 +2748,7 @@
       <c r="H14" t="s">
         <v>21</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="I14" s="3" t="s">
         <v>127</v>
       </c>
       <c r="J14" t="s">
@@ -2581,7 +2777,7 @@
       <c r="C15" t="s">
         <v>131</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="5">
         <v>46162</v>
       </c>
       <c r="E15" t="s">
@@ -2596,7 +2792,7 @@
       <c r="H15" t="s">
         <v>21</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="I15" s="3" t="s">
         <v>133</v>
       </c>
       <c r="J15" t="s">
@@ -2622,10 +2818,10 @@
       <c r="B16" t="s">
         <v>136</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="5">
         <v>46163</v>
       </c>
       <c r="E16" t="s">
@@ -2640,7 +2836,7 @@
       <c r="H16" t="s">
         <v>21</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="3" t="s">
         <v>139</v>
       </c>
       <c r="J16" t="s">
@@ -2673,7 +2869,7 @@
     <hyperlink ref="C12" r:id="rId10" display="https://dlc.sh/lernangebot/6599?lz=47"/>
     <hyperlink ref="C13" r:id="rId11" display="https://dlc.sh/lernangebot/859?lz=101"/>
     <hyperlink ref="C14" r:id="rId12" display="https://dlc.sh/lernangebot/6779?lz=122"/>
-    <hyperlink ref="C16" r:id="rId13" display="https://dlc.sh/lernangebot/6733?lz=112"/>
+    <hyperlink ref="C16" r:id="rId13" display="https://dlc.sh/lernangebot/6733?lz=112" tooltip="https://dlc.sh/lernangebot/6733?lz=112"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -2890,7 +3086,7 @@
       <c r="E10" t="s">
         <v>191</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="3" t="s">
         <v>192</v>
       </c>
     </row>
@@ -2978,4 +3174,341 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:N7"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14" outlineLevelRow="6"/>
+  <cols>
+    <col min="2" max="2" width="60.1818181818182" customWidth="1"/>
+    <col min="3" max="3" width="46" customWidth="1"/>
+    <col min="4" max="4" width="19.4545454545455" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7272727272727" customWidth="1"/>
+    <col min="6" max="6" width="12.0909090909091" customWidth="1"/>
+    <col min="7" max="7" width="13.1818181818182" customWidth="1"/>
+    <col min="8" max="8" width="10.3636363636364" customWidth="1"/>
+    <col min="9" max="9" width="17.2727272727273" customWidth="1"/>
+    <col min="10" max="10" width="44.8181818181818" customWidth="1"/>
+    <col min="11" max="11" width="40.2727272727273" customWidth="1"/>
+    <col min="12" max="12" width="28.7272727272727" customWidth="1"/>
+    <col min="13" max="13" width="13.5454545454545" customWidth="1"/>
+    <col min="14" max="14" width="46" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C1" t="s">
+        <v>215</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>216</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>217</v>
+      </c>
+      <c r="L1" t="s">
+        <v>218</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="2" ht="50" customHeight="1" spans="1:14">
+      <c r="A2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D2" s="1">
+        <v>46185</v>
+      </c>
+      <c r="E2" t="s">
+        <v>223</v>
+      </c>
+      <c r="F2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="M2" t="s">
+        <v>228</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="3" ht="50" customHeight="1" spans="1:14">
+      <c r="A3" t="s">
+        <v>230</v>
+      </c>
+      <c r="B3" t="s">
+        <v>231</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="D3" s="1">
+        <v>46191</v>
+      </c>
+      <c r="E3" t="s">
+        <v>233</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
+        <v>234</v>
+      </c>
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="M3" t="s">
+        <v>228</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1" spans="1:14">
+      <c r="A4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="C4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D4" s="1">
+        <v>46193</v>
+      </c>
+      <c r="E4" t="s">
+        <v>242</v>
+      </c>
+      <c r="F4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="M4" t="s">
+        <v>228</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1" spans="1:14">
+      <c r="A5" t="s">
+        <v>247</v>
+      </c>
+      <c r="B5" t="s">
+        <v>248</v>
+      </c>
+      <c r="C5" t="s">
+        <v>249</v>
+      </c>
+      <c r="D5" s="1">
+        <v>46197</v>
+      </c>
+      <c r="E5" t="s">
+        <v>250</v>
+      </c>
+      <c r="F5" t="s">
+        <v>96</v>
+      </c>
+      <c r="G5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="M5" t="s">
+        <v>228</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1" spans="1:14">
+      <c r="A6" t="s">
+        <v>255</v>
+      </c>
+      <c r="B6" t="s">
+        <v>256</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="D6" s="1">
+        <v>46199</v>
+      </c>
+      <c r="E6" t="s">
+        <v>258</v>
+      </c>
+      <c r="F6" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="M6" t="s">
+        <v>228</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1" spans="1:14">
+      <c r="A7" t="s">
+        <v>263</v>
+      </c>
+      <c r="B7" t="s">
+        <v>264</v>
+      </c>
+      <c r="C7" t="s">
+        <v>265</v>
+      </c>
+      <c r="F7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G7" t="s">
+        <v>234</v>
+      </c>
+      <c r="H7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="M7" t="s">
+        <v>228</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" display="https://dlc.sh/" tooltip="https://dlc.sh/"/>
+    <hyperlink ref="I3" r:id="rId1" display="https://dlc.sh/" tooltip="https://dlc.sh/"/>
+    <hyperlink ref="I4" r:id="rId1" display="https://dlc.sh/" tooltip="https://dlc.sh/"/>
+    <hyperlink ref="I5" r:id="rId1" display="https://dlc.sh/" tooltip="https://dlc.sh/"/>
+    <hyperlink ref="I6" r:id="rId1" display="https://dlc.sh/" tooltip="https://dlc.sh/"/>
+    <hyperlink ref="I7" r:id="rId1" display="https://dlc.sh/" tooltip="https://dlc.sh/"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>